<commit_message>
Documentacion completa de pruebas unitarias
</commit_message>
<xml_diff>
--- a/Doc_Test/Pruebas_Calidad/Pruebas_Unitarias/CEC-1.xlsx
+++ b/Doc_Test/Pruebas_Calidad/Pruebas_Unitarias/CEC-1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\Desktop\Resultados_Test\Pruebas_Calidad\Pruebas_Unitarias\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\Desktop\App_Uv\AppAcompanhamientoUV\Doc_Test\Pruebas_Calidad\Pruebas_Unitarias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A9BC572-1604-42EC-84A0-DB809631EB17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE61F65B-F26E-4CFD-B831-050B79933DA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2FFDA8E8-6428-4D51-9D6D-F314F8731DBF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="264">
   <si>
     <t>ID</t>
   </si>
@@ -844,6 +844,12 @@
   </si>
   <si>
     <t>(1) El usuario debe ingresar todos los campos solicitados para registrar correctamente el usuario, en caso de dejar una casilla en blanco se le debe alertar.                                                                                                                                           (2) El usuario debe ingresar un rut válido, en caso de no ingresarlo se le debe alertar.                                                       (3) El usuario debe ingresar un correo válido, en caso de no ingresarlo se le debe alertar.                                                 (4) El usuario debe ingresar un número telefónico válido, en caso de no ingresarlo se le debe alertar.                                                                                    (5) La contraseña ingresada debe cumplir con el mínimo de exigencia en seguridad, de caso contrario se le solicitará que modifique su contraseña.                                                                                                                                                             (6) No se pueden registrar 2 usuario con el mismo correo.                                                                                                      (7) No se pueden registrar 2 usuarios con el mismo Rut.</t>
+  </si>
+  <si>
+    <t>Aprobado  con observaciones</t>
+  </si>
+  <si>
+    <t>Ausencia de pestaña de carga que indique el usuario debe esperar tras presionar el botón, al no mostrar nada se puede intuir que no funciona correctamente.</t>
   </si>
 </sst>
 </file>
@@ -1052,12 +1058,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1090,6 +1090,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1447,127 +1453,127 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
     </row>
     <row r="4" spans="2:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="25"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="24">
         <v>45841</v>
       </c>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="26"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="24"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
     </row>
     <row r="7" spans="2:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
-      <c r="J8" s="24"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
     </row>
     <row r="9" spans="2:10" ht="127.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="27" t="s">
         <v>261</v>
       </c>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="29"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
     </row>
     <row r="10" spans="2:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="28"/>
+      <c r="C10" s="26"/>
       <c r="D10" s="6" t="s">
         <v>6</v>
       </c>
@@ -1625,10 +1631,10 @@
       <c r="H12" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="I12" s="19" t="s">
+      <c r="I12" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="J12" s="19"/>
+      <c r="J12" s="17"/>
     </row>
     <row r="13" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B13" s="14"/>
@@ -1650,11 +1656,11 @@
       <c r="H13" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="I13" s="20"/>
-      <c r="J13" s="20"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="19" t="s">
         <v>28</v>
       </c>
       <c r="C14" s="15" t="s">
@@ -1669,7 +1675,7 @@
       <c r="J14" s="15"/>
     </row>
     <row r="15" spans="2:10" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="22"/>
+      <c r="B15" s="20"/>
       <c r="C15" s="7" t="s">
         <v>29</v>
       </c>
@@ -1696,7 +1702,7 @@
       </c>
     </row>
     <row r="16" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B16" s="22"/>
+      <c r="B16" s="20"/>
       <c r="C16" s="9" t="s">
         <v>30</v>
       </c>
@@ -1719,7 +1725,7 @@
       <c r="J16" s="16"/>
     </row>
     <row r="17" spans="2:10" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B17" s="22"/>
+      <c r="B17" s="20"/>
       <c r="C17" s="9" t="s">
         <v>36</v>
       </c>
@@ -1742,7 +1748,7 @@
       <c r="J17" s="16"/>
     </row>
     <row r="18" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B18" s="22"/>
+      <c r="B18" s="20"/>
       <c r="C18" s="7" t="s">
         <v>39</v>
       </c>
@@ -1765,7 +1771,7 @@
       <c r="J18" s="16"/>
     </row>
     <row r="19" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B19" s="22"/>
+      <c r="B19" s="20"/>
       <c r="C19" s="9" t="s">
         <v>53</v>
       </c>
@@ -1788,7 +1794,7 @@
       <c r="J19" s="16"/>
     </row>
     <row r="20" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B20" s="22"/>
+      <c r="B20" s="20"/>
       <c r="C20" s="9" t="s">
         <v>54</v>
       </c>
@@ -1811,7 +1817,7 @@
       <c r="J20" s="16"/>
     </row>
     <row r="21" spans="2:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="22"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="7" t="s">
         <v>55</v>
       </c>
@@ -1834,7 +1840,7 @@
       <c r="J21" s="16"/>
     </row>
     <row r="22" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B22" s="22"/>
+      <c r="B22" s="20"/>
       <c r="C22" s="9" t="s">
         <v>56</v>
       </c>
@@ -1857,7 +1863,7 @@
       <c r="J22" s="16"/>
     </row>
     <row r="23" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B23" s="22"/>
+      <c r="B23" s="20"/>
       <c r="C23" s="9" t="s">
         <v>57</v>
       </c>
@@ -1880,7 +1886,7 @@
       <c r="J23" s="16"/>
     </row>
     <row r="24" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B24" s="22"/>
+      <c r="B24" s="20"/>
       <c r="C24" s="7" t="s">
         <v>58</v>
       </c>
@@ -1903,7 +1909,7 @@
       <c r="J24" s="16"/>
     </row>
     <row r="25" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B25" s="23"/>
+      <c r="B25" s="21"/>
       <c r="C25" s="9" t="s">
         <v>59</v>
       </c>
@@ -1926,7 +1932,7 @@
       <c r="J25" s="16"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="28" t="s">
         <v>52</v>
       </c>
       <c r="C26" s="15" t="s">
@@ -1941,7 +1947,7 @@
       <c r="J26" s="15"/>
     </row>
     <row r="27" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B27" s="18"/>
+      <c r="B27" s="28"/>
       <c r="C27" s="7" t="s">
         <v>70</v>
       </c>
@@ -1968,7 +1974,7 @@
       </c>
     </row>
     <row r="28" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B28" s="18"/>
+      <c r="B28" s="28"/>
       <c r="C28" s="9" t="s">
         <v>71</v>
       </c>
@@ -1991,7 +1997,7 @@
       <c r="J28" s="16"/>
     </row>
     <row r="29" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B29" s="18"/>
+      <c r="B29" s="28"/>
       <c r="C29" s="9" t="s">
         <v>72</v>
       </c>
@@ -2014,7 +2020,7 @@
       <c r="J29" s="16"/>
     </row>
     <row r="30" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B30" s="18"/>
+      <c r="B30" s="28"/>
       <c r="C30" s="9" t="s">
         <v>73</v>
       </c>
@@ -2037,7 +2043,7 @@
       <c r="J30" s="16"/>
     </row>
     <row r="31" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B31" s="18"/>
+      <c r="B31" s="28"/>
       <c r="C31" s="9" t="s">
         <v>74</v>
       </c>
@@ -2060,7 +2066,7 @@
       <c r="J31" s="16"/>
     </row>
     <row r="32" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B32" s="18"/>
+      <c r="B32" s="28"/>
       <c r="C32" s="9" t="s">
         <v>75</v>
       </c>
@@ -2083,7 +2089,7 @@
       <c r="J32" s="16"/>
     </row>
     <row r="33" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B33" s="18"/>
+      <c r="B33" s="28"/>
       <c r="C33" s="9" t="s">
         <v>76</v>
       </c>
@@ -2105,8 +2111,8 @@
       <c r="I33" s="16"/>
       <c r="J33" s="16"/>
     </row>
-    <row r="34" spans="2:10" ht="144" x14ac:dyDescent="0.3">
-      <c r="B34" s="18"/>
+    <row r="34" spans="2:10" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="B34" s="28"/>
       <c r="C34" s="9" t="s">
         <v>77</v>
       </c>
@@ -2129,7 +2135,7 @@
       <c r="J34" s="16"/>
     </row>
     <row r="35" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B35" s="18"/>
+      <c r="B35" s="28"/>
       <c r="C35" s="9" t="s">
         <v>78</v>
       </c>
@@ -3586,10 +3592,10 @@
       <c r="H99" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I99" s="17" t="s">
+      <c r="I99" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="J99" s="17"/>
+      <c r="J99" s="29"/>
     </row>
     <row r="100" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B100" s="14"/>
@@ -3611,8 +3617,8 @@
       <c r="H100" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I100" s="17"/>
-      <c r="J100" s="17"/>
+      <c r="I100" s="29"/>
+      <c r="J100" s="29"/>
     </row>
     <row r="101" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B101" s="14"/>
@@ -3634,8 +3640,8 @@
       <c r="H101" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I101" s="17"/>
-      <c r="J101" s="17"/>
+      <c r="I101" s="29"/>
+      <c r="J101" s="29"/>
     </row>
     <row r="102" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B102" s="14"/>
@@ -3657,8 +3663,8 @@
       <c r="H102" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I102" s="17"/>
-      <c r="J102" s="17"/>
+      <c r="I102" s="29"/>
+      <c r="J102" s="29"/>
     </row>
     <row r="103" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B103" s="14"/>
@@ -3680,8 +3686,8 @@
       <c r="H103" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I103" s="17"/>
-      <c r="J103" s="17"/>
+      <c r="I103" s="29"/>
+      <c r="J103" s="29"/>
     </row>
     <row r="104" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B104" s="14"/>
@@ -3703,8 +3709,8 @@
       <c r="H104" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I104" s="17"/>
-      <c r="J104" s="17"/>
+      <c r="I104" s="29"/>
+      <c r="J104" s="29"/>
     </row>
     <row r="105" spans="2:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B105" s="14"/>
@@ -3726,8 +3732,8 @@
       <c r="H105" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I105" s="17"/>
-      <c r="J105" s="17"/>
+      <c r="I105" s="29"/>
+      <c r="J105" s="29"/>
     </row>
     <row r="106" spans="2:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B106" s="14"/>
@@ -3749,8 +3755,8 @@
       <c r="H106" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I106" s="17"/>
-      <c r="J106" s="17"/>
+      <c r="I106" s="29"/>
+      <c r="J106" s="29"/>
     </row>
     <row r="107" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B107" s="14"/>
@@ -3772,8 +3778,8 @@
       <c r="H107" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I107" s="17"/>
-      <c r="J107" s="17"/>
+      <c r="I107" s="29"/>
+      <c r="J107" s="29"/>
     </row>
     <row r="108" spans="2:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B108" s="14"/>
@@ -3795,8 +3801,8 @@
       <c r="H108" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I108" s="17"/>
-      <c r="J108" s="17"/>
+      <c r="I108" s="29"/>
+      <c r="J108" s="29"/>
     </row>
     <row r="109" spans="2:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B109" s="14"/>
@@ -3818,8 +3824,8 @@
       <c r="H109" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I109" s="17"/>
-      <c r="J109" s="17"/>
+      <c r="I109" s="29"/>
+      <c r="J109" s="29"/>
     </row>
     <row r="110" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B110" s="14" t="s">
@@ -4677,7 +4683,7 @@
       <c r="I147" s="16"/>
       <c r="J147" s="16"/>
     </row>
-    <row r="148" spans="2:10" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B148" s="14"/>
       <c r="C148" s="9" t="s">
         <v>246</v>
@@ -4924,7 +4930,7 @@
       <c r="I158" s="16"/>
       <c r="J158" s="16"/>
     </row>
-    <row r="159" spans="2:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:10" ht="331.2" x14ac:dyDescent="0.3">
       <c r="B159" s="14"/>
       <c r="C159" s="9" t="s">
         <v>246</v>
@@ -5171,7 +5177,7 @@
       <c r="I169" s="16"/>
       <c r="J169" s="16"/>
     </row>
-    <row r="170" spans="2:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:10" ht="331.2" x14ac:dyDescent="0.3">
       <c r="B170" s="14"/>
       <c r="C170" s="9" t="s">
         <v>246</v>
@@ -5230,9 +5236,11 @@
         <v>25</v>
       </c>
       <c r="I172" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="J172" s="16"/>
+        <v>262</v>
+      </c>
+      <c r="J172" s="16" t="s">
+        <v>263</v>
+      </c>
     </row>
     <row r="173" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B173" s="14"/>
@@ -5418,7 +5426,7 @@
       <c r="I180" s="16"/>
       <c r="J180" s="16"/>
     </row>
-    <row r="181" spans="2:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:10" ht="331.2" x14ac:dyDescent="0.3">
       <c r="B181" s="14"/>
       <c r="C181" s="9" t="s">
         <v>246</v>
@@ -5443,14 +5451,56 @@
     </row>
   </sheetData>
   <mergeCells count="73">
-    <mergeCell ref="B160:B170"/>
-    <mergeCell ref="C160:J160"/>
-    <mergeCell ref="I161:I170"/>
-    <mergeCell ref="J161:J170"/>
-    <mergeCell ref="B171:B181"/>
-    <mergeCell ref="C171:J171"/>
-    <mergeCell ref="I172:I181"/>
-    <mergeCell ref="J172:J181"/>
+    <mergeCell ref="B138:B148"/>
+    <mergeCell ref="C138:J138"/>
+    <mergeCell ref="I139:I148"/>
+    <mergeCell ref="J139:J148"/>
+    <mergeCell ref="B149:B159"/>
+    <mergeCell ref="C149:J149"/>
+    <mergeCell ref="I150:I159"/>
+    <mergeCell ref="J150:J159"/>
+    <mergeCell ref="B110:B119"/>
+    <mergeCell ref="C110:J110"/>
+    <mergeCell ref="I111:I119"/>
+    <mergeCell ref="J111:J119"/>
+    <mergeCell ref="C120:J120"/>
+    <mergeCell ref="B120:B137"/>
+    <mergeCell ref="I121:I137"/>
+    <mergeCell ref="J121:J137"/>
+    <mergeCell ref="C98:J98"/>
+    <mergeCell ref="B98:B109"/>
+    <mergeCell ref="I99:I109"/>
+    <mergeCell ref="J99:J109"/>
+    <mergeCell ref="C89:J89"/>
+    <mergeCell ref="B89:B97"/>
+    <mergeCell ref="I90:I97"/>
+    <mergeCell ref="J90:J97"/>
+    <mergeCell ref="B79:B88"/>
+    <mergeCell ref="C79:J79"/>
+    <mergeCell ref="I80:I88"/>
+    <mergeCell ref="J80:J88"/>
+    <mergeCell ref="B62:B69"/>
+    <mergeCell ref="C62:J62"/>
+    <mergeCell ref="I63:I69"/>
+    <mergeCell ref="J63:J69"/>
+    <mergeCell ref="B70:B78"/>
+    <mergeCell ref="C70:J70"/>
+    <mergeCell ref="I71:I78"/>
+    <mergeCell ref="J71:J78"/>
+    <mergeCell ref="I37:I48"/>
+    <mergeCell ref="J37:J48"/>
+    <mergeCell ref="B36:B48"/>
+    <mergeCell ref="B49:B61"/>
+    <mergeCell ref="C49:J49"/>
+    <mergeCell ref="I50:I61"/>
+    <mergeCell ref="J50:J61"/>
+    <mergeCell ref="C36:J36"/>
+    <mergeCell ref="C26:J26"/>
+    <mergeCell ref="I27:I35"/>
+    <mergeCell ref="J27:J35"/>
+    <mergeCell ref="B26:B35"/>
+    <mergeCell ref="I15:I25"/>
+    <mergeCell ref="J15:J25"/>
     <mergeCell ref="C14:J14"/>
     <mergeCell ref="I12:I13"/>
     <mergeCell ref="J12:J13"/>
@@ -5466,56 +5516,14 @@
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="C9:J9"/>
     <mergeCell ref="C11:J11"/>
-    <mergeCell ref="C26:J26"/>
-    <mergeCell ref="I27:I35"/>
-    <mergeCell ref="J27:J35"/>
-    <mergeCell ref="B26:B35"/>
-    <mergeCell ref="I15:I25"/>
-    <mergeCell ref="J15:J25"/>
-    <mergeCell ref="I37:I48"/>
-    <mergeCell ref="J37:J48"/>
-    <mergeCell ref="B36:B48"/>
-    <mergeCell ref="B49:B61"/>
-    <mergeCell ref="C49:J49"/>
-    <mergeCell ref="I50:I61"/>
-    <mergeCell ref="J50:J61"/>
-    <mergeCell ref="C36:J36"/>
-    <mergeCell ref="B79:B88"/>
-    <mergeCell ref="C79:J79"/>
-    <mergeCell ref="I80:I88"/>
-    <mergeCell ref="J80:J88"/>
-    <mergeCell ref="B62:B69"/>
-    <mergeCell ref="C62:J62"/>
-    <mergeCell ref="I63:I69"/>
-    <mergeCell ref="J63:J69"/>
-    <mergeCell ref="B70:B78"/>
-    <mergeCell ref="C70:J70"/>
-    <mergeCell ref="I71:I78"/>
-    <mergeCell ref="J71:J78"/>
-    <mergeCell ref="C98:J98"/>
-    <mergeCell ref="B98:B109"/>
-    <mergeCell ref="I99:I109"/>
-    <mergeCell ref="J99:J109"/>
-    <mergeCell ref="C89:J89"/>
-    <mergeCell ref="B89:B97"/>
-    <mergeCell ref="I90:I97"/>
-    <mergeCell ref="J90:J97"/>
-    <mergeCell ref="B110:B119"/>
-    <mergeCell ref="C110:J110"/>
-    <mergeCell ref="I111:I119"/>
-    <mergeCell ref="J111:J119"/>
-    <mergeCell ref="C120:J120"/>
-    <mergeCell ref="B120:B137"/>
-    <mergeCell ref="I121:I137"/>
-    <mergeCell ref="J121:J137"/>
-    <mergeCell ref="B138:B148"/>
-    <mergeCell ref="C138:J138"/>
-    <mergeCell ref="I139:I148"/>
-    <mergeCell ref="J139:J148"/>
-    <mergeCell ref="B149:B159"/>
-    <mergeCell ref="C149:J149"/>
-    <mergeCell ref="I150:I159"/>
-    <mergeCell ref="J150:J159"/>
+    <mergeCell ref="B160:B170"/>
+    <mergeCell ref="C160:J160"/>
+    <mergeCell ref="I161:I170"/>
+    <mergeCell ref="J161:J170"/>
+    <mergeCell ref="B171:B181"/>
+    <mergeCell ref="C171:J171"/>
+    <mergeCell ref="I172:I181"/>
+    <mergeCell ref="J172:J181"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E54" r:id="rId1" xr:uid="{F6F46655-4BB2-4006-8068-9345E4CC6ADA}"/>

</xml_diff>